<commit_message>
Cleaned and standardized the data.
</commit_message>
<xml_diff>
--- a/Sleep_health_and_lifestyle_dataset.xlsx
+++ b/Sleep_health_and_lifestyle_dataset.xlsx
@@ -5,18 +5,29 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Learning\Datasets\Sleep_health_and_lifestyle_dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Learning\Projects\Power BI\Sleep, Health, &amp; Lifestyle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CA04283-5168-4D53-8B0C-A9BE8C294D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE2CCB8-38DC-4FEC-891D-B8A90BD74900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{6425CDAD-B65E-4412-85DF-C3C1E3683B73}"/>
+    <workbookView minimized="1" xWindow="6150" yWindow="3015" windowWidth="21600" windowHeight="11835" xr2:uid="{6425CDAD-B65E-4412-85DF-C3C1E3683B73}"/>
   </bookViews>
   <sheets>
     <sheet name="Sleep_health_and_lifestyle_data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>

</xml_diff>